<commit_message>
Updates to Database classes for ph_cis ph_trans properties and optimized state labeler and .xlsx metadata sheets updated
</commit_message>
<xml_diff>
--- a/database/PeptideDatabase-70_mv_F427A_guesthost_peptides.xlsx
+++ b/database/PeptideDatabase-70_mv_F427A_guesthost_peptides.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bakrantz/Documents/python/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7967C24-E99E-594E-A46B-1E518160A142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{287B3748-0F46-4942-84B1-613A19FD3039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{771C88DF-88B2-E348-BE11-2567F4397102}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="300">
   <si>
     <t>guesthost_Ala</t>
   </si>
@@ -919,6 +919,21 @@
   </si>
   <si>
     <t>11o14001-guesthost_Ala-70_mV-F427A-400_Hz-downsampled-rpt_2.csv</t>
+  </si>
+  <si>
+    <t>ph_cis</t>
+  </si>
+  <si>
+    <t>ph_trans</t>
+  </si>
+  <si>
+    <t>salt</t>
+  </si>
+  <si>
+    <t>salt_conc</t>
+  </si>
+  <si>
+    <t>KCl</t>
   </si>
 </sst>
 </file>
@@ -1823,7 +1838,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBB02983-7886-F046-AB34-426E7E084EE9}">
-  <dimension ref="A1:Y93"/>
+  <dimension ref="A1:AC93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" bestFit="1" customWidth="1"/>
@@ -1836,14 +1851,18 @@
     <col min="9" max="9" width="14.5" customWidth="1"/>
     <col min="10" max="10" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.5" customWidth="1"/>
-    <col min="15" max="15" width="62" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.5" customWidth="1"/>
+    <col min="19" max="19" width="62" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>7</v>
       </c>
@@ -1878,21 +1897,33 @@
         <v>24</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="T1" s="1"/>
-      <c r="Y1" s="1"/>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="X1" s="1"/>
+      <c r="AC1" s="1"/>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1926,16 +1957,28 @@
         <v>25</v>
       </c>
       <c r="L2">
+        <v>5.6</v>
+      </c>
+      <c r="M2">
+        <v>5.6</v>
+      </c>
+      <c r="N2" t="s">
+        <v>299</v>
+      </c>
+      <c r="O2">
+        <v>0.1</v>
+      </c>
+      <c r="P2">
         <v>20</v>
       </c>
-      <c r="M2">
+      <c r="Q2">
         <v>600</v>
       </c>
-      <c r="O2" t="s">
+      <c r="S2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1969,16 +2012,28 @@
         <v>25</v>
       </c>
       <c r="L3">
+        <v>5.6</v>
+      </c>
+      <c r="M3">
+        <v>5.6</v>
+      </c>
+      <c r="N3" t="s">
+        <v>299</v>
+      </c>
+      <c r="O3">
+        <v>0.1</v>
+      </c>
+      <c r="P3">
         <v>20</v>
       </c>
-      <c r="M3">
+      <c r="Q3">
         <v>600</v>
       </c>
-      <c r="O3" t="s">
+      <c r="S3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -2012,16 +2067,28 @@
         <v>25</v>
       </c>
       <c r="L4">
+        <v>5.6</v>
+      </c>
+      <c r="M4">
+        <v>5.6</v>
+      </c>
+      <c r="N4" t="s">
+        <v>299</v>
+      </c>
+      <c r="O4">
+        <v>0.1</v>
+      </c>
+      <c r="P4">
         <v>20</v>
       </c>
-      <c r="M4">
+      <c r="Q4">
         <v>600</v>
       </c>
-      <c r="O4" t="s">
+      <c r="S4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -2055,16 +2122,28 @@
         <v>25</v>
       </c>
       <c r="L5">
+        <v>5.6</v>
+      </c>
+      <c r="M5">
+        <v>5.6</v>
+      </c>
+      <c r="N5" t="s">
+        <v>299</v>
+      </c>
+      <c r="O5">
+        <v>0.1</v>
+      </c>
+      <c r="P5">
         <v>20</v>
       </c>
-      <c r="M5">
+      <c r="Q5">
         <v>600</v>
       </c>
-      <c r="O5" t="s">
+      <c r="S5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -2098,16 +2177,28 @@
         <v>25</v>
       </c>
       <c r="L6">
+        <v>5.6</v>
+      </c>
+      <c r="M6">
+        <v>5.6</v>
+      </c>
+      <c r="N6" t="s">
+        <v>299</v>
+      </c>
+      <c r="O6">
+        <v>0.1</v>
+      </c>
+      <c r="P6">
         <v>20</v>
       </c>
-      <c r="M6">
+      <c r="Q6">
         <v>600</v>
       </c>
-      <c r="O6" t="s">
+      <c r="S6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -2141,16 +2232,28 @@
         <v>25</v>
       </c>
       <c r="L7">
+        <v>5.6</v>
+      </c>
+      <c r="M7">
+        <v>5.6</v>
+      </c>
+      <c r="N7" t="s">
+        <v>299</v>
+      </c>
+      <c r="O7">
+        <v>0.1</v>
+      </c>
+      <c r="P7">
         <v>20</v>
       </c>
-      <c r="M7">
+      <c r="Q7">
         <v>600</v>
       </c>
-      <c r="O7" t="s">
+      <c r="S7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -2184,16 +2287,28 @@
         <v>25</v>
       </c>
       <c r="L8">
+        <v>5.6</v>
+      </c>
+      <c r="M8">
+        <v>5.6</v>
+      </c>
+      <c r="N8" t="s">
+        <v>299</v>
+      </c>
+      <c r="O8">
+        <v>0.1</v>
+      </c>
+      <c r="P8">
         <v>20</v>
       </c>
-      <c r="M8">
+      <c r="Q8">
         <v>600</v>
       </c>
-      <c r="O8" t="s">
+      <c r="S8" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -2227,16 +2342,28 @@
         <v>25</v>
       </c>
       <c r="L9">
+        <v>5.6</v>
+      </c>
+      <c r="M9">
+        <v>5.6</v>
+      </c>
+      <c r="N9" t="s">
+        <v>299</v>
+      </c>
+      <c r="O9">
+        <v>0.1</v>
+      </c>
+      <c r="P9">
         <v>20</v>
       </c>
-      <c r="M9">
+      <c r="Q9">
         <v>600</v>
       </c>
-      <c r="O9" t="s">
+      <c r="S9" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -2270,16 +2397,28 @@
         <v>25</v>
       </c>
       <c r="L10">
+        <v>5.6</v>
+      </c>
+      <c r="M10">
+        <v>5.6</v>
+      </c>
+      <c r="N10" t="s">
+        <v>299</v>
+      </c>
+      <c r="O10">
+        <v>0.1</v>
+      </c>
+      <c r="P10">
         <v>20</v>
       </c>
-      <c r="M10">
+      <c r="Q10">
         <v>400</v>
       </c>
-      <c r="O10" t="s">
+      <c r="S10" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -2313,16 +2452,28 @@
         <v>25</v>
       </c>
       <c r="L11">
+        <v>5.6</v>
+      </c>
+      <c r="M11">
+        <v>5.6</v>
+      </c>
+      <c r="N11" t="s">
+        <v>299</v>
+      </c>
+      <c r="O11">
+        <v>0.1</v>
+      </c>
+      <c r="P11">
         <v>20</v>
       </c>
-      <c r="M11">
+      <c r="Q11">
         <v>400</v>
       </c>
-      <c r="O11" t="s">
+      <c r="S11" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -2356,16 +2507,28 @@
         <v>25</v>
       </c>
       <c r="L12">
+        <v>5.6</v>
+      </c>
+      <c r="M12">
+        <v>5.6</v>
+      </c>
+      <c r="N12" t="s">
+        <v>299</v>
+      </c>
+      <c r="O12">
+        <v>0.1</v>
+      </c>
+      <c r="P12">
         <v>20</v>
       </c>
-      <c r="M12">
+      <c r="Q12">
         <v>400</v>
       </c>
-      <c r="O12" t="s">
+      <c r="S12" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -2399,16 +2562,28 @@
         <v>25</v>
       </c>
       <c r="L13">
+        <v>5.6</v>
+      </c>
+      <c r="M13">
+        <v>5.6</v>
+      </c>
+      <c r="N13" t="s">
+        <v>299</v>
+      </c>
+      <c r="O13">
+        <v>0.1</v>
+      </c>
+      <c r="P13">
         <v>20</v>
       </c>
-      <c r="M13">
+      <c r="Q13">
         <v>400</v>
       </c>
-      <c r="O13" t="s">
+      <c r="S13" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -2442,16 +2617,28 @@
         <v>25</v>
       </c>
       <c r="L14">
+        <v>5.6</v>
+      </c>
+      <c r="M14">
+        <v>5.6</v>
+      </c>
+      <c r="N14" t="s">
+        <v>299</v>
+      </c>
+      <c r="O14">
+        <v>0.1</v>
+      </c>
+      <c r="P14">
         <v>20</v>
       </c>
-      <c r="M14">
+      <c r="Q14">
         <v>400</v>
       </c>
-      <c r="O14" t="s">
+      <c r="S14" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -2485,16 +2672,28 @@
         <v>25</v>
       </c>
       <c r="L15">
+        <v>5.6</v>
+      </c>
+      <c r="M15">
+        <v>5.6</v>
+      </c>
+      <c r="N15" t="s">
+        <v>299</v>
+      </c>
+      <c r="O15">
+        <v>0.1</v>
+      </c>
+      <c r="P15">
         <v>20</v>
       </c>
-      <c r="M15">
+      <c r="Q15">
         <v>400</v>
       </c>
-      <c r="O15" t="s">
+      <c r="S15" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -2528,16 +2727,28 @@
         <v>25</v>
       </c>
       <c r="L16">
+        <v>5.6</v>
+      </c>
+      <c r="M16">
+        <v>5.6</v>
+      </c>
+      <c r="N16" t="s">
+        <v>299</v>
+      </c>
+      <c r="O16">
+        <v>0.1</v>
+      </c>
+      <c r="P16">
         <v>20</v>
       </c>
-      <c r="M16">
+      <c r="Q16">
         <v>400</v>
       </c>
-      <c r="O16" t="s">
+      <c r="S16" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -2571,16 +2782,28 @@
         <v>25</v>
       </c>
       <c r="L17">
+        <v>5.6</v>
+      </c>
+      <c r="M17">
+        <v>5.6</v>
+      </c>
+      <c r="N17" t="s">
+        <v>299</v>
+      </c>
+      <c r="O17">
+        <v>0.1</v>
+      </c>
+      <c r="P17">
         <v>20</v>
       </c>
-      <c r="M17">
+      <c r="Q17">
         <v>400</v>
       </c>
-      <c r="O17" t="s">
+      <c r="S17" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="18" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>1</v>
       </c>
@@ -2613,17 +2836,29 @@
       <c r="K18" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L18" s="6">
+      <c r="L18">
+        <v>5.6</v>
+      </c>
+      <c r="M18">
+        <v>5.6</v>
+      </c>
+      <c r="N18" t="s">
+        <v>299</v>
+      </c>
+      <c r="O18">
+        <v>0.1</v>
+      </c>
+      <c r="P18" s="6">
         <v>20</v>
       </c>
-      <c r="M18" s="6">
+      <c r="Q18" s="6">
         <v>600</v>
       </c>
-      <c r="O18" s="6" t="s">
+      <c r="S18" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>1</v>
       </c>
@@ -2656,17 +2891,29 @@
       <c r="K19" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L19" s="6">
+      <c r="L19">
+        <v>5.6</v>
+      </c>
+      <c r="M19">
+        <v>5.6</v>
+      </c>
+      <c r="N19" t="s">
+        <v>299</v>
+      </c>
+      <c r="O19">
+        <v>0.1</v>
+      </c>
+      <c r="P19" s="6">
         <v>20</v>
       </c>
-      <c r="M19" s="6">
+      <c r="Q19" s="6">
         <v>600</v>
       </c>
-      <c r="O19" s="6" t="s">
+      <c r="S19" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>1</v>
       </c>
@@ -2699,17 +2946,29 @@
       <c r="K20" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L20" s="6">
+      <c r="L20">
+        <v>5.6</v>
+      </c>
+      <c r="M20">
+        <v>5.6</v>
+      </c>
+      <c r="N20" t="s">
+        <v>299</v>
+      </c>
+      <c r="O20">
+        <v>0.1</v>
+      </c>
+      <c r="P20" s="6">
         <v>20</v>
       </c>
-      <c r="M20" s="6">
+      <c r="Q20" s="6">
         <v>600</v>
       </c>
-      <c r="O20" s="6" t="s">
+      <c r="S20" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
         <v>1</v>
       </c>
@@ -2742,17 +3001,29 @@
       <c r="K21" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L21" s="6">
+      <c r="L21">
+        <v>5.6</v>
+      </c>
+      <c r="M21">
+        <v>5.6</v>
+      </c>
+      <c r="N21" t="s">
+        <v>299</v>
+      </c>
+      <c r="O21">
+        <v>0.1</v>
+      </c>
+      <c r="P21" s="6">
         <v>20</v>
       </c>
-      <c r="M21" s="6">
+      <c r="Q21" s="6">
         <v>600</v>
       </c>
-      <c r="O21" s="6" t="s">
+      <c r="S21" s="6" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>1</v>
       </c>
@@ -2785,17 +3056,29 @@
       <c r="K22" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L22" s="6">
+      <c r="L22">
+        <v>5.6</v>
+      </c>
+      <c r="M22">
+        <v>5.6</v>
+      </c>
+      <c r="N22" t="s">
+        <v>299</v>
+      </c>
+      <c r="O22">
+        <v>0.1</v>
+      </c>
+      <c r="P22" s="6">
         <v>20</v>
       </c>
-      <c r="M22" s="6">
+      <c r="Q22" s="6">
         <v>600</v>
       </c>
-      <c r="O22" s="6" t="s">
+      <c r="S22" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
         <v>1</v>
       </c>
@@ -2828,17 +3111,29 @@
       <c r="K23" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L23" s="6">
+      <c r="L23">
+        <v>5.6</v>
+      </c>
+      <c r="M23">
+        <v>5.6</v>
+      </c>
+      <c r="N23" t="s">
+        <v>299</v>
+      </c>
+      <c r="O23">
+        <v>0.1</v>
+      </c>
+      <c r="P23" s="6">
         <v>20</v>
       </c>
-      <c r="M23" s="6">
+      <c r="Q23" s="6">
         <v>600</v>
       </c>
-      <c r="O23" s="6" t="s">
+      <c r="S23" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
         <v>1</v>
       </c>
@@ -2871,17 +3166,29 @@
       <c r="K24" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L24" s="6">
+      <c r="L24">
+        <v>5.6</v>
+      </c>
+      <c r="M24">
+        <v>5.6</v>
+      </c>
+      <c r="N24" t="s">
+        <v>299</v>
+      </c>
+      <c r="O24">
+        <v>0.1</v>
+      </c>
+      <c r="P24" s="6">
         <v>20</v>
       </c>
-      <c r="M24" s="6">
+      <c r="Q24" s="6">
         <v>400</v>
       </c>
-      <c r="O24" s="6" t="s">
+      <c r="S24" s="6" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="25" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>1</v>
       </c>
@@ -2914,17 +3221,29 @@
       <c r="K25" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L25" s="6">
+      <c r="L25">
+        <v>5.6</v>
+      </c>
+      <c r="M25">
+        <v>5.6</v>
+      </c>
+      <c r="N25" t="s">
+        <v>299</v>
+      </c>
+      <c r="O25">
+        <v>0.1</v>
+      </c>
+      <c r="P25" s="6">
         <v>20</v>
       </c>
-      <c r="M25" s="6">
+      <c r="Q25" s="6">
         <v>400</v>
       </c>
-      <c r="O25" s="6" t="s">
+      <c r="S25" s="6" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
         <v>1</v>
       </c>
@@ -2957,17 +3276,29 @@
       <c r="K26" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L26" s="6">
+      <c r="L26">
+        <v>5.6</v>
+      </c>
+      <c r="M26">
+        <v>5.6</v>
+      </c>
+      <c r="N26" t="s">
+        <v>299</v>
+      </c>
+      <c r="O26">
+        <v>0.1</v>
+      </c>
+      <c r="P26" s="6">
         <v>20</v>
       </c>
-      <c r="M26" s="6">
+      <c r="Q26" s="6">
         <v>400</v>
       </c>
-      <c r="O26" s="6" t="s">
+      <c r="S26" s="6" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="27" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
         <v>1</v>
       </c>
@@ -3000,17 +3331,29 @@
       <c r="K27" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L27" s="6">
+      <c r="L27">
+        <v>5.6</v>
+      </c>
+      <c r="M27">
+        <v>5.6</v>
+      </c>
+      <c r="N27" t="s">
+        <v>299</v>
+      </c>
+      <c r="O27">
+        <v>0.1</v>
+      </c>
+      <c r="P27" s="6">
         <v>20</v>
       </c>
-      <c r="M27" s="6">
+      <c r="Q27" s="6">
         <v>400</v>
       </c>
-      <c r="O27" s="6" t="s">
+      <c r="S27" s="6" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="28" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
         <v>1</v>
       </c>
@@ -3043,17 +3386,29 @@
       <c r="K28" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L28" s="6">
+      <c r="L28">
+        <v>5.6</v>
+      </c>
+      <c r="M28">
+        <v>5.6</v>
+      </c>
+      <c r="N28" t="s">
+        <v>299</v>
+      </c>
+      <c r="O28">
+        <v>0.1</v>
+      </c>
+      <c r="P28" s="6">
         <v>20</v>
       </c>
-      <c r="M28" s="6">
+      <c r="Q28" s="6">
         <v>400</v>
       </c>
-      <c r="O28" s="6" t="s">
+      <c r="S28" s="6" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="29" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
         <v>1</v>
       </c>
@@ -3086,17 +3441,29 @@
       <c r="K29" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L29" s="6">
+      <c r="L29">
+        <v>5.6</v>
+      </c>
+      <c r="M29">
+        <v>5.6</v>
+      </c>
+      <c r="N29" t="s">
+        <v>299</v>
+      </c>
+      <c r="O29">
+        <v>0.1</v>
+      </c>
+      <c r="P29" s="6">
         <v>20</v>
       </c>
-      <c r="M29" s="6">
+      <c r="Q29" s="6">
         <v>400</v>
       </c>
-      <c r="O29" s="6" t="s">
+      <c r="S29" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -3130,16 +3497,28 @@
         <v>25</v>
       </c>
       <c r="L30">
+        <v>5.6</v>
+      </c>
+      <c r="M30">
+        <v>5.6</v>
+      </c>
+      <c r="N30" t="s">
+        <v>299</v>
+      </c>
+      <c r="O30">
+        <v>0.1</v>
+      </c>
+      <c r="P30">
         <v>20</v>
       </c>
-      <c r="M30">
+      <c r="Q30">
         <v>600</v>
       </c>
-      <c r="O30" t="s">
+      <c r="S30" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>2</v>
       </c>
@@ -3173,16 +3552,28 @@
         <v>25</v>
       </c>
       <c r="L31">
+        <v>5.6</v>
+      </c>
+      <c r="M31">
+        <v>5.6</v>
+      </c>
+      <c r="N31" t="s">
+        <v>299</v>
+      </c>
+      <c r="O31">
+        <v>0.1</v>
+      </c>
+      <c r="P31">
         <v>20</v>
       </c>
-      <c r="M31">
+      <c r="Q31">
         <v>600</v>
       </c>
-      <c r="O31" t="s">
+      <c r="S31" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>2</v>
       </c>
@@ -3216,16 +3607,28 @@
         <v>25</v>
       </c>
       <c r="L32">
+        <v>5.6</v>
+      </c>
+      <c r="M32">
+        <v>5.6</v>
+      </c>
+      <c r="N32" t="s">
+        <v>299</v>
+      </c>
+      <c r="O32">
+        <v>0.1</v>
+      </c>
+      <c r="P32">
         <v>20</v>
       </c>
-      <c r="M32">
+      <c r="Q32">
         <v>600</v>
       </c>
-      <c r="O32" t="s">
+      <c r="S32" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>2</v>
       </c>
@@ -3259,16 +3662,28 @@
         <v>25</v>
       </c>
       <c r="L33">
+        <v>5.6</v>
+      </c>
+      <c r="M33">
+        <v>5.6</v>
+      </c>
+      <c r="N33" t="s">
+        <v>299</v>
+      </c>
+      <c r="O33">
+        <v>0.1</v>
+      </c>
+      <c r="P33">
         <v>20</v>
       </c>
-      <c r="M33">
+      <c r="Q33">
         <v>600</v>
       </c>
-      <c r="O33" t="s">
+      <c r="S33" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -3302,16 +3717,28 @@
         <v>25</v>
       </c>
       <c r="L34">
+        <v>5.6</v>
+      </c>
+      <c r="M34">
+        <v>5.6</v>
+      </c>
+      <c r="N34" t="s">
+        <v>299</v>
+      </c>
+      <c r="O34">
+        <v>0.1</v>
+      </c>
+      <c r="P34">
         <v>20</v>
       </c>
-      <c r="M34">
+      <c r="Q34">
         <v>600</v>
       </c>
-      <c r="O34" t="s">
+      <c r="S34" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>2</v>
       </c>
@@ -3345,16 +3772,28 @@
         <v>25</v>
       </c>
       <c r="L35">
+        <v>5.6</v>
+      </c>
+      <c r="M35">
+        <v>5.6</v>
+      </c>
+      <c r="N35" t="s">
+        <v>299</v>
+      </c>
+      <c r="O35">
+        <v>0.1</v>
+      </c>
+      <c r="P35">
         <v>20</v>
       </c>
-      <c r="M35">
+      <c r="Q35">
         <v>600</v>
       </c>
-      <c r="O35" t="s">
+      <c r="S35" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>2</v>
       </c>
@@ -3388,16 +3827,28 @@
         <v>25</v>
       </c>
       <c r="L36">
+        <v>5.6</v>
+      </c>
+      <c r="M36">
+        <v>5.6</v>
+      </c>
+      <c r="N36" t="s">
+        <v>299</v>
+      </c>
+      <c r="O36">
+        <v>0.1</v>
+      </c>
+      <c r="P36">
         <v>20</v>
       </c>
-      <c r="M36">
+      <c r="Q36">
         <v>400</v>
       </c>
-      <c r="O36" t="s">
+      <c r="S36" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>2</v>
       </c>
@@ -3431,16 +3882,28 @@
         <v>25</v>
       </c>
       <c r="L37">
+        <v>5.6</v>
+      </c>
+      <c r="M37">
+        <v>5.6</v>
+      </c>
+      <c r="N37" t="s">
+        <v>299</v>
+      </c>
+      <c r="O37">
+        <v>0.1</v>
+      </c>
+      <c r="P37">
         <v>20</v>
       </c>
-      <c r="M37">
+      <c r="Q37">
         <v>400</v>
       </c>
-      <c r="O37" t="s">
+      <c r="S37" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -3474,16 +3937,28 @@
         <v>25</v>
       </c>
       <c r="L38">
+        <v>5.6</v>
+      </c>
+      <c r="M38">
+        <v>5.6</v>
+      </c>
+      <c r="N38" t="s">
+        <v>299</v>
+      </c>
+      <c r="O38">
+        <v>0.1</v>
+      </c>
+      <c r="P38">
         <v>20</v>
       </c>
-      <c r="M38">
+      <c r="Q38">
         <v>400</v>
       </c>
-      <c r="O38" t="s">
+      <c r="S38" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>2</v>
       </c>
@@ -3517,16 +3992,28 @@
         <v>25</v>
       </c>
       <c r="L39">
+        <v>5.6</v>
+      </c>
+      <c r="M39">
+        <v>5.6</v>
+      </c>
+      <c r="N39" t="s">
+        <v>299</v>
+      </c>
+      <c r="O39">
+        <v>0.1</v>
+      </c>
+      <c r="P39">
         <v>20</v>
       </c>
-      <c r="M39">
+      <c r="Q39">
         <v>400</v>
       </c>
-      <c r="O39" t="s">
+      <c r="S39" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>2</v>
       </c>
@@ -3560,16 +4047,28 @@
         <v>25</v>
       </c>
       <c r="L40">
+        <v>5.6</v>
+      </c>
+      <c r="M40">
+        <v>5.6</v>
+      </c>
+      <c r="N40" t="s">
+        <v>299</v>
+      </c>
+      <c r="O40">
+        <v>0.1</v>
+      </c>
+      <c r="P40">
         <v>20</v>
       </c>
-      <c r="M40">
+      <c r="Q40">
         <v>400</v>
       </c>
-      <c r="O40" t="s">
+      <c r="S40" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>2</v>
       </c>
@@ -3603,16 +4102,28 @@
         <v>25</v>
       </c>
       <c r="L41">
+        <v>5.6</v>
+      </c>
+      <c r="M41">
+        <v>5.6</v>
+      </c>
+      <c r="N41" t="s">
+        <v>299</v>
+      </c>
+      <c r="O41">
+        <v>0.1</v>
+      </c>
+      <c r="P41">
         <v>20</v>
       </c>
-      <c r="M41">
+      <c r="Q41">
         <v>400</v>
       </c>
-      <c r="O41" t="s">
+      <c r="S41" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="42" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
         <v>3</v>
       </c>
@@ -3645,17 +4156,29 @@
       <c r="K42" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L42" s="6">
+      <c r="L42">
+        <v>5.6</v>
+      </c>
+      <c r="M42">
+        <v>5.6</v>
+      </c>
+      <c r="N42" t="s">
+        <v>299</v>
+      </c>
+      <c r="O42">
+        <v>0.1</v>
+      </c>
+      <c r="P42" s="6">
         <v>20</v>
       </c>
-      <c r="M42" s="6">
+      <c r="Q42" s="6">
         <v>500</v>
       </c>
-      <c r="O42" s="6" t="s">
+      <c r="S42" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="43" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
         <v>3</v>
       </c>
@@ -3688,17 +4211,29 @@
       <c r="K43" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L43" s="6">
+      <c r="L43">
+        <v>5.6</v>
+      </c>
+      <c r="M43">
+        <v>5.6</v>
+      </c>
+      <c r="N43" t="s">
+        <v>299</v>
+      </c>
+      <c r="O43">
+        <v>0.1</v>
+      </c>
+      <c r="P43" s="6">
         <v>20</v>
       </c>
-      <c r="M43" s="6">
+      <c r="Q43" s="6">
         <v>500</v>
       </c>
-      <c r="O43" s="6" t="s">
+      <c r="S43" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="44" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
         <v>3</v>
       </c>
@@ -3731,17 +4266,29 @@
       <c r="K44" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L44" s="6">
+      <c r="L44">
+        <v>5.6</v>
+      </c>
+      <c r="M44">
+        <v>5.6</v>
+      </c>
+      <c r="N44" t="s">
+        <v>299</v>
+      </c>
+      <c r="O44">
+        <v>0.1</v>
+      </c>
+      <c r="P44" s="6">
         <v>20</v>
       </c>
-      <c r="M44" s="6">
+      <c r="Q44" s="6">
         <v>500</v>
       </c>
-      <c r="O44" s="6" t="s">
+      <c r="S44" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="45" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="6" t="s">
         <v>3</v>
       </c>
@@ -3774,17 +4321,29 @@
       <c r="K45" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L45" s="6">
+      <c r="L45">
+        <v>5.6</v>
+      </c>
+      <c r="M45">
+        <v>5.6</v>
+      </c>
+      <c r="N45" t="s">
+        <v>299</v>
+      </c>
+      <c r="O45">
+        <v>0.1</v>
+      </c>
+      <c r="P45" s="6">
         <v>20</v>
       </c>
-      <c r="M45" s="6">
+      <c r="Q45" s="6">
         <v>500</v>
       </c>
-      <c r="O45" s="6" t="s">
+      <c r="S45" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="46" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
         <v>3</v>
       </c>
@@ -3817,17 +4376,29 @@
       <c r="K46" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L46" s="6">
+      <c r="L46">
+        <v>5.6</v>
+      </c>
+      <c r="M46">
+        <v>5.6</v>
+      </c>
+      <c r="N46" t="s">
+        <v>299</v>
+      </c>
+      <c r="O46">
+        <v>0.1</v>
+      </c>
+      <c r="P46" s="6">
         <v>20</v>
       </c>
-      <c r="M46" s="6">
+      <c r="Q46" s="6">
         <v>500</v>
       </c>
-      <c r="O46" s="6" t="s">
+      <c r="S46" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="47" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
         <v>3</v>
       </c>
@@ -3860,17 +4431,29 @@
       <c r="K47" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L47" s="6">
+      <c r="L47">
+        <v>5.6</v>
+      </c>
+      <c r="M47">
+        <v>5.6</v>
+      </c>
+      <c r="N47" t="s">
+        <v>299</v>
+      </c>
+      <c r="O47">
+        <v>0.1</v>
+      </c>
+      <c r="P47" s="6">
         <v>20</v>
       </c>
-      <c r="M47" s="6">
+      <c r="Q47" s="6">
         <v>500</v>
       </c>
-      <c r="O47" s="6" t="s">
+      <c r="S47" s="6" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="48" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
         <v>3</v>
       </c>
@@ -3903,17 +4486,29 @@
       <c r="K48" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L48" s="6">
+      <c r="L48">
+        <v>5.6</v>
+      </c>
+      <c r="M48">
+        <v>5.6</v>
+      </c>
+      <c r="N48" t="s">
+        <v>299</v>
+      </c>
+      <c r="O48">
+        <v>0.1</v>
+      </c>
+      <c r="P48" s="6">
         <v>20</v>
       </c>
-      <c r="M48" s="6">
+      <c r="Q48" s="6">
         <v>400</v>
       </c>
-      <c r="O48" s="6" t="s">
+      <c r="S48" s="6" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="49" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
         <v>3</v>
       </c>
@@ -3946,17 +4541,29 @@
       <c r="K49" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L49" s="6">
+      <c r="L49">
+        <v>5.6</v>
+      </c>
+      <c r="M49">
+        <v>5.6</v>
+      </c>
+      <c r="N49" t="s">
+        <v>299</v>
+      </c>
+      <c r="O49">
+        <v>0.1</v>
+      </c>
+      <c r="P49" s="6">
         <v>20</v>
       </c>
-      <c r="M49" s="6">
+      <c r="Q49" s="6">
         <v>400</v>
       </c>
-      <c r="O49" s="6" t="s">
+      <c r="S49" s="6" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="50" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="6" t="s">
         <v>3</v>
       </c>
@@ -3989,17 +4596,29 @@
       <c r="K50" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L50" s="6">
+      <c r="L50">
+        <v>5.6</v>
+      </c>
+      <c r="M50">
+        <v>5.6</v>
+      </c>
+      <c r="N50" t="s">
+        <v>299</v>
+      </c>
+      <c r="O50">
+        <v>0.1</v>
+      </c>
+      <c r="P50" s="6">
         <v>20</v>
       </c>
-      <c r="M50" s="6">
+      <c r="Q50" s="6">
         <v>400</v>
       </c>
-      <c r="O50" s="6" t="s">
+      <c r="S50" s="6" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="51" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
         <v>3</v>
       </c>
@@ -4032,17 +4651,29 @@
       <c r="K51" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L51" s="6">
+      <c r="L51">
+        <v>5.6</v>
+      </c>
+      <c r="M51">
+        <v>5.6</v>
+      </c>
+      <c r="N51" t="s">
+        <v>299</v>
+      </c>
+      <c r="O51">
+        <v>0.1</v>
+      </c>
+      <c r="P51" s="6">
         <v>20</v>
       </c>
-      <c r="M51" s="6">
+      <c r="Q51" s="6">
         <v>400</v>
       </c>
-      <c r="O51" s="6" t="s">
+      <c r="S51" s="6" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="52" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
         <v>3</v>
       </c>
@@ -4075,17 +4706,29 @@
       <c r="K52" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L52" s="6">
+      <c r="L52">
+        <v>5.6</v>
+      </c>
+      <c r="M52">
+        <v>5.6</v>
+      </c>
+      <c r="N52" t="s">
+        <v>299</v>
+      </c>
+      <c r="O52">
+        <v>0.1</v>
+      </c>
+      <c r="P52" s="6">
         <v>20</v>
       </c>
-      <c r="M52" s="6">
+      <c r="Q52" s="6">
         <v>400</v>
       </c>
-      <c r="O52" s="6" t="s">
+      <c r="S52" s="6" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="53" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="6" t="s">
         <v>3</v>
       </c>
@@ -4118,17 +4761,29 @@
       <c r="K53" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L53" s="6">
+      <c r="L53">
+        <v>5.6</v>
+      </c>
+      <c r="M53">
+        <v>5.6</v>
+      </c>
+      <c r="N53" t="s">
+        <v>299</v>
+      </c>
+      <c r="O53">
+        <v>0.1</v>
+      </c>
+      <c r="P53" s="6">
         <v>20</v>
       </c>
-      <c r="M53" s="6">
+      <c r="Q53" s="6">
         <v>400</v>
       </c>
-      <c r="O53" s="6" t="s">
+      <c r="S53" s="6" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>4</v>
       </c>
@@ -4162,16 +4817,28 @@
         <v>25</v>
       </c>
       <c r="L54">
+        <v>5.6</v>
+      </c>
+      <c r="M54">
+        <v>5.6</v>
+      </c>
+      <c r="N54" t="s">
+        <v>299</v>
+      </c>
+      <c r="O54">
+        <v>0.1</v>
+      </c>
+      <c r="P54">
         <v>18</v>
       </c>
-      <c r="M54">
+      <c r="Q54">
         <v>500</v>
       </c>
-      <c r="O54" t="s">
+      <c r="S54" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>4</v>
       </c>
@@ -4205,16 +4872,28 @@
         <v>25</v>
       </c>
       <c r="L55">
+        <v>5.6</v>
+      </c>
+      <c r="M55">
+        <v>5.6</v>
+      </c>
+      <c r="N55" t="s">
+        <v>299</v>
+      </c>
+      <c r="O55">
+        <v>0.1</v>
+      </c>
+      <c r="P55">
         <v>18</v>
       </c>
-      <c r="M55">
+      <c r="Q55">
         <v>500</v>
       </c>
-      <c r="O55" t="s">
+      <c r="S55" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>4</v>
       </c>
@@ -4248,16 +4927,28 @@
         <v>25</v>
       </c>
       <c r="L56">
+        <v>5.6</v>
+      </c>
+      <c r="M56">
+        <v>5.6</v>
+      </c>
+      <c r="N56" t="s">
+        <v>299</v>
+      </c>
+      <c r="O56">
+        <v>0.1</v>
+      </c>
+      <c r="P56">
         <v>18</v>
       </c>
-      <c r="M56">
+      <c r="Q56">
         <v>500</v>
       </c>
-      <c r="O56" t="s">
+      <c r="S56" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>4</v>
       </c>
@@ -4291,16 +4982,28 @@
         <v>25</v>
       </c>
       <c r="L57">
+        <v>5.6</v>
+      </c>
+      <c r="M57">
+        <v>5.6</v>
+      </c>
+      <c r="N57" t="s">
+        <v>299</v>
+      </c>
+      <c r="O57">
+        <v>0.1</v>
+      </c>
+      <c r="P57">
         <v>18</v>
       </c>
-      <c r="M57">
+      <c r="Q57">
         <v>400</v>
       </c>
-      <c r="O57" t="s">
+      <c r="S57" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>4</v>
       </c>
@@ -4334,16 +5037,28 @@
         <v>25</v>
       </c>
       <c r="L58">
+        <v>5.6</v>
+      </c>
+      <c r="M58">
+        <v>5.6</v>
+      </c>
+      <c r="N58" t="s">
+        <v>299</v>
+      </c>
+      <c r="O58">
+        <v>0.1</v>
+      </c>
+      <c r="P58">
         <v>18</v>
       </c>
-      <c r="M58">
+      <c r="Q58">
         <v>400</v>
       </c>
-      <c r="O58" t="s">
+      <c r="S58" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>4</v>
       </c>
@@ -4377,16 +5092,28 @@
         <v>25</v>
       </c>
       <c r="L59">
+        <v>5.6</v>
+      </c>
+      <c r="M59">
+        <v>5.6</v>
+      </c>
+      <c r="N59" t="s">
+        <v>299</v>
+      </c>
+      <c r="O59">
+        <v>0.1</v>
+      </c>
+      <c r="P59">
         <v>18</v>
       </c>
-      <c r="M59">
+      <c r="Q59">
         <v>400</v>
       </c>
-      <c r="O59" t="s">
+      <c r="S59" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="60" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
         <v>5</v>
       </c>
@@ -4419,17 +5146,29 @@
       <c r="K60" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L60" s="6">
+      <c r="L60">
+        <v>5.6</v>
+      </c>
+      <c r="M60">
+        <v>5.6</v>
+      </c>
+      <c r="N60" t="s">
+        <v>299</v>
+      </c>
+      <c r="O60">
+        <v>0.1</v>
+      </c>
+      <c r="P60" s="6">
         <v>19</v>
       </c>
-      <c r="M60" s="6">
+      <c r="Q60" s="6">
         <v>600</v>
       </c>
-      <c r="O60" s="6" t="s">
+      <c r="S60" s="6" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="61" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A61" s="6" t="s">
         <v>5</v>
       </c>
@@ -4462,17 +5201,29 @@
       <c r="K61" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L61" s="6">
+      <c r="L61">
+        <v>5.6</v>
+      </c>
+      <c r="M61">
+        <v>5.6</v>
+      </c>
+      <c r="N61" t="s">
+        <v>299</v>
+      </c>
+      <c r="O61">
+        <v>0.1</v>
+      </c>
+      <c r="P61" s="6">
         <v>19</v>
       </c>
-      <c r="M61" s="6">
+      <c r="Q61" s="6">
         <v>600</v>
       </c>
-      <c r="O61" s="6" t="s">
+      <c r="S61" s="6" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="62" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="6" t="s">
         <v>5</v>
       </c>
@@ -4505,17 +5256,29 @@
       <c r="K62" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L62" s="6">
+      <c r="L62">
+        <v>5.6</v>
+      </c>
+      <c r="M62">
+        <v>5.6</v>
+      </c>
+      <c r="N62" t="s">
+        <v>299</v>
+      </c>
+      <c r="O62">
+        <v>0.1</v>
+      </c>
+      <c r="P62" s="6">
         <v>19</v>
       </c>
-      <c r="M62" s="6">
+      <c r="Q62" s="6">
         <v>600</v>
       </c>
-      <c r="O62" s="6" t="s">
+      <c r="S62" s="6" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="63" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="6" t="s">
         <v>5</v>
       </c>
@@ -4548,17 +5311,29 @@
       <c r="K63" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L63" s="6">
+      <c r="L63">
+        <v>5.6</v>
+      </c>
+      <c r="M63">
+        <v>5.6</v>
+      </c>
+      <c r="N63" t="s">
+        <v>299</v>
+      </c>
+      <c r="O63">
+        <v>0.1</v>
+      </c>
+      <c r="P63" s="6">
         <v>19</v>
       </c>
-      <c r="M63" s="6">
+      <c r="Q63" s="6">
         <v>600</v>
       </c>
-      <c r="O63" s="6" t="s">
+      <c r="S63" s="6" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="64" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="6" t="s">
         <v>5</v>
       </c>
@@ -4591,17 +5366,29 @@
       <c r="K64" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L64" s="6">
+      <c r="L64">
+        <v>5.6</v>
+      </c>
+      <c r="M64">
+        <v>5.6</v>
+      </c>
+      <c r="N64" t="s">
+        <v>299</v>
+      </c>
+      <c r="O64">
+        <v>0.1</v>
+      </c>
+      <c r="P64" s="6">
         <v>19</v>
       </c>
-      <c r="M64" s="6">
+      <c r="Q64" s="6">
         <v>600</v>
       </c>
-      <c r="O64" s="6" t="s">
+      <c r="S64" s="6" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="65" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A65" s="6" t="s">
         <v>5</v>
       </c>
@@ -4634,17 +5421,29 @@
       <c r="K65" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L65" s="6">
+      <c r="L65">
+        <v>5.6</v>
+      </c>
+      <c r="M65">
+        <v>5.6</v>
+      </c>
+      <c r="N65" t="s">
+        <v>299</v>
+      </c>
+      <c r="O65">
+        <v>0.1</v>
+      </c>
+      <c r="P65" s="6">
         <v>19</v>
       </c>
-      <c r="M65" s="6">
+      <c r="Q65" s="6">
         <v>600</v>
       </c>
-      <c r="O65" s="6" t="s">
+      <c r="S65" s="6" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="66" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="6" t="s">
         <v>5</v>
       </c>
@@ -4677,17 +5476,29 @@
       <c r="K66" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L66" s="6">
+      <c r="L66">
+        <v>5.6</v>
+      </c>
+      <c r="M66">
+        <v>5.6</v>
+      </c>
+      <c r="N66" t="s">
+        <v>299</v>
+      </c>
+      <c r="O66">
+        <v>0.1</v>
+      </c>
+      <c r="P66" s="6">
         <v>19</v>
       </c>
-      <c r="M66" s="6">
+      <c r="Q66" s="6">
         <v>600</v>
       </c>
-      <c r="O66" s="6" t="s">
+      <c r="S66" s="6" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="67" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
         <v>5</v>
       </c>
@@ -4720,17 +5531,29 @@
       <c r="K67" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L67" s="6">
+      <c r="L67">
+        <v>5.6</v>
+      </c>
+      <c r="M67">
+        <v>5.6</v>
+      </c>
+      <c r="N67" t="s">
+        <v>299</v>
+      </c>
+      <c r="O67">
+        <v>0.1</v>
+      </c>
+      <c r="P67" s="6">
         <v>19</v>
       </c>
-      <c r="M67" s="6">
+      <c r="Q67" s="6">
         <v>600</v>
       </c>
-      <c r="O67" s="6" t="s">
+      <c r="S67" s="6" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="68" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
         <v>5</v>
       </c>
@@ -4763,17 +5586,29 @@
       <c r="K68" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L68" s="6">
+      <c r="L68">
+        <v>5.6</v>
+      </c>
+      <c r="M68">
+        <v>5.6</v>
+      </c>
+      <c r="N68" t="s">
+        <v>299</v>
+      </c>
+      <c r="O68">
+        <v>0.1</v>
+      </c>
+      <c r="P68" s="6">
         <v>19</v>
       </c>
-      <c r="M68" s="6">
+      <c r="Q68" s="6">
         <v>400</v>
       </c>
-      <c r="O68" s="6" t="s">
+      <c r="S68" s="6" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="69" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
         <v>5</v>
       </c>
@@ -4806,17 +5641,29 @@
       <c r="K69" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L69" s="6">
+      <c r="L69">
+        <v>5.6</v>
+      </c>
+      <c r="M69">
+        <v>5.6</v>
+      </c>
+      <c r="N69" t="s">
+        <v>299</v>
+      </c>
+      <c r="O69">
+        <v>0.1</v>
+      </c>
+      <c r="P69" s="6">
         <v>19</v>
       </c>
-      <c r="M69" s="6">
+      <c r="Q69" s="6">
         <v>400</v>
       </c>
-      <c r="O69" s="6" t="s">
+      <c r="S69" s="6" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="70" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
         <v>5</v>
       </c>
@@ -4849,17 +5696,29 @@
       <c r="K70" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L70" s="6">
+      <c r="L70">
+        <v>5.6</v>
+      </c>
+      <c r="M70">
+        <v>5.6</v>
+      </c>
+      <c r="N70" t="s">
+        <v>299</v>
+      </c>
+      <c r="O70">
+        <v>0.1</v>
+      </c>
+      <c r="P70" s="6">
         <v>19</v>
       </c>
-      <c r="M70" s="6">
+      <c r="Q70" s="6">
         <v>400</v>
       </c>
-      <c r="O70" s="6" t="s">
+      <c r="S70" s="6" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="71" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
         <v>5</v>
       </c>
@@ -4892,17 +5751,29 @@
       <c r="K71" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L71" s="6">
+      <c r="L71">
+        <v>5.6</v>
+      </c>
+      <c r="M71">
+        <v>5.6</v>
+      </c>
+      <c r="N71" t="s">
+        <v>299</v>
+      </c>
+      <c r="O71">
+        <v>0.1</v>
+      </c>
+      <c r="P71" s="6">
         <v>19</v>
       </c>
-      <c r="M71" s="6">
+      <c r="Q71" s="6">
         <v>400</v>
       </c>
-      <c r="O71" s="6" t="s">
+      <c r="S71" s="6" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="72" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
         <v>5</v>
       </c>
@@ -4935,17 +5806,29 @@
       <c r="K72" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L72" s="6">
+      <c r="L72">
+        <v>5.6</v>
+      </c>
+      <c r="M72">
+        <v>5.6</v>
+      </c>
+      <c r="N72" t="s">
+        <v>299</v>
+      </c>
+      <c r="O72">
+        <v>0.1</v>
+      </c>
+      <c r="P72" s="6">
         <v>19</v>
       </c>
-      <c r="M72" s="6">
+      <c r="Q72" s="6">
         <v>400</v>
       </c>
-      <c r="O72" s="6" t="s">
+      <c r="S72" s="6" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="73" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="6" t="s">
         <v>5</v>
       </c>
@@ -4978,17 +5861,29 @@
       <c r="K73" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L73" s="6">
+      <c r="L73">
+        <v>5.6</v>
+      </c>
+      <c r="M73">
+        <v>5.6</v>
+      </c>
+      <c r="N73" t="s">
+        <v>299</v>
+      </c>
+      <c r="O73">
+        <v>0.1</v>
+      </c>
+      <c r="P73" s="6">
         <v>19</v>
       </c>
-      <c r="M73" s="6">
+      <c r="Q73" s="6">
         <v>400</v>
       </c>
-      <c r="O73" s="6" t="s">
+      <c r="S73" s="6" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="74" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
         <v>5</v>
       </c>
@@ -5021,17 +5916,29 @@
       <c r="K74" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L74" s="6">
+      <c r="L74">
+        <v>5.6</v>
+      </c>
+      <c r="M74">
+        <v>5.6</v>
+      </c>
+      <c r="N74" t="s">
+        <v>299</v>
+      </c>
+      <c r="O74">
+        <v>0.1</v>
+      </c>
+      <c r="P74" s="6">
         <v>19</v>
       </c>
-      <c r="M74" s="6">
+      <c r="Q74" s="6">
         <v>400</v>
       </c>
-      <c r="O74" s="6" t="s">
+      <c r="S74" s="6" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="75" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A75" s="6" t="s">
         <v>5</v>
       </c>
@@ -5064,17 +5971,29 @@
       <c r="K75" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L75" s="6">
+      <c r="L75">
+        <v>5.6</v>
+      </c>
+      <c r="M75">
+        <v>5.6</v>
+      </c>
+      <c r="N75" t="s">
+        <v>299</v>
+      </c>
+      <c r="O75">
+        <v>0.1</v>
+      </c>
+      <c r="P75" s="6">
         <v>19</v>
       </c>
-      <c r="M75" s="6">
+      <c r="Q75" s="6">
         <v>400</v>
       </c>
-      <c r="O75" s="6" t="s">
+      <c r="S75" s="6" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>6</v>
       </c>
@@ -5108,16 +6027,28 @@
         <v>25</v>
       </c>
       <c r="L76">
+        <v>5.6</v>
+      </c>
+      <c r="M76">
+        <v>5.6</v>
+      </c>
+      <c r="N76" t="s">
+        <v>299</v>
+      </c>
+      <c r="O76">
+        <v>0.1</v>
+      </c>
+      <c r="P76">
         <v>20</v>
       </c>
-      <c r="M76">
+      <c r="Q76">
         <v>600</v>
       </c>
-      <c r="O76" t="s">
+      <c r="S76" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>6</v>
       </c>
@@ -5151,16 +6082,28 @@
         <v>25</v>
       </c>
       <c r="L77">
+        <v>5.6</v>
+      </c>
+      <c r="M77">
+        <v>5.6</v>
+      </c>
+      <c r="N77" t="s">
+        <v>299</v>
+      </c>
+      <c r="O77">
+        <v>0.1</v>
+      </c>
+      <c r="P77">
         <v>20</v>
       </c>
-      <c r="M77">
+      <c r="Q77">
         <v>600</v>
       </c>
-      <c r="O77" t="s">
+      <c r="S77" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>6</v>
       </c>
@@ -5194,16 +6137,28 @@
         <v>25</v>
       </c>
       <c r="L78">
+        <v>5.6</v>
+      </c>
+      <c r="M78">
+        <v>5.6</v>
+      </c>
+      <c r="N78" t="s">
+        <v>299</v>
+      </c>
+      <c r="O78">
+        <v>0.1</v>
+      </c>
+      <c r="P78">
         <v>20</v>
       </c>
-      <c r="M78">
+      <c r="Q78">
         <v>600</v>
       </c>
-      <c r="O78" t="s">
+      <c r="S78" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>6</v>
       </c>
@@ -5237,16 +6192,28 @@
         <v>25</v>
       </c>
       <c r="L79">
+        <v>5.6</v>
+      </c>
+      <c r="M79">
+        <v>5.6</v>
+      </c>
+      <c r="N79" t="s">
+        <v>299</v>
+      </c>
+      <c r="O79">
+        <v>0.1</v>
+      </c>
+      <c r="P79">
         <v>20</v>
       </c>
-      <c r="M79">
+      <c r="Q79">
         <v>600</v>
       </c>
-      <c r="O79" t="s">
+      <c r="S79" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>6</v>
       </c>
@@ -5280,16 +6247,28 @@
         <v>25</v>
       </c>
       <c r="L80">
+        <v>5.6</v>
+      </c>
+      <c r="M80">
+        <v>5.6</v>
+      </c>
+      <c r="N80" t="s">
+        <v>299</v>
+      </c>
+      <c r="O80">
+        <v>0.1</v>
+      </c>
+      <c r="P80">
         <v>20</v>
       </c>
-      <c r="M80">
+      <c r="Q80">
         <v>600</v>
       </c>
-      <c r="O80" t="s">
+      <c r="S80" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>6</v>
       </c>
@@ -5323,16 +6302,28 @@
         <v>25</v>
       </c>
       <c r="L81">
+        <v>5.6</v>
+      </c>
+      <c r="M81">
+        <v>5.6</v>
+      </c>
+      <c r="N81" t="s">
+        <v>299</v>
+      </c>
+      <c r="O81">
+        <v>0.1</v>
+      </c>
+      <c r="P81">
         <v>179</v>
       </c>
-      <c r="M81">
+      <c r="Q81">
         <v>600</v>
       </c>
-      <c r="O81" t="s">
+      <c r="S81" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>6</v>
       </c>
@@ -5366,16 +6357,28 @@
         <v>25</v>
       </c>
       <c r="L82">
+        <v>5.6</v>
+      </c>
+      <c r="M82">
+        <v>5.6</v>
+      </c>
+      <c r="N82" t="s">
+        <v>299</v>
+      </c>
+      <c r="O82">
+        <v>0.1</v>
+      </c>
+      <c r="P82">
         <v>179</v>
       </c>
-      <c r="M82">
+      <c r="Q82">
         <v>600</v>
       </c>
-      <c r="O82" t="s">
+      <c r="S82" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>6</v>
       </c>
@@ -5409,16 +6412,28 @@
         <v>25</v>
       </c>
       <c r="L83">
+        <v>5.6</v>
+      </c>
+      <c r="M83">
+        <v>5.6</v>
+      </c>
+      <c r="N83" t="s">
+        <v>299</v>
+      </c>
+      <c r="O83">
+        <v>0.1</v>
+      </c>
+      <c r="P83">
         <v>179</v>
       </c>
-      <c r="M83">
+      <c r="Q83">
         <v>600</v>
       </c>
-      <c r="O83" t="s">
+      <c r="S83" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>6</v>
       </c>
@@ -5452,16 +6467,28 @@
         <v>25</v>
       </c>
       <c r="L84">
+        <v>5.6</v>
+      </c>
+      <c r="M84">
+        <v>5.6</v>
+      </c>
+      <c r="N84" t="s">
+        <v>299</v>
+      </c>
+      <c r="O84">
+        <v>0.1</v>
+      </c>
+      <c r="P84">
         <v>179</v>
       </c>
-      <c r="M84">
+      <c r="Q84">
         <v>600</v>
       </c>
-      <c r="O84" t="s">
+      <c r="S84" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>6</v>
       </c>
@@ -5495,16 +6522,28 @@
         <v>25</v>
       </c>
       <c r="L85">
+        <v>5.6</v>
+      </c>
+      <c r="M85">
+        <v>5.6</v>
+      </c>
+      <c r="N85" t="s">
+        <v>299</v>
+      </c>
+      <c r="O85">
+        <v>0.1</v>
+      </c>
+      <c r="P85">
         <v>20</v>
       </c>
-      <c r="M85">
+      <c r="Q85">
         <v>400</v>
       </c>
-      <c r="O85" t="s">
+      <c r="S85" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>6</v>
       </c>
@@ -5538,16 +6577,28 @@
         <v>25</v>
       </c>
       <c r="L86">
+        <v>5.6</v>
+      </c>
+      <c r="M86">
+        <v>5.6</v>
+      </c>
+      <c r="N86" t="s">
+        <v>299</v>
+      </c>
+      <c r="O86">
+        <v>0.1</v>
+      </c>
+      <c r="P86">
         <v>20</v>
       </c>
-      <c r="M86">
+      <c r="Q86">
         <v>400</v>
       </c>
-      <c r="O86" t="s">
+      <c r="S86" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>6</v>
       </c>
@@ -5581,16 +6632,28 @@
         <v>25</v>
       </c>
       <c r="L87">
+        <v>5.6</v>
+      </c>
+      <c r="M87">
+        <v>5.6</v>
+      </c>
+      <c r="N87" t="s">
+        <v>299</v>
+      </c>
+      <c r="O87">
+        <v>0.1</v>
+      </c>
+      <c r="P87">
         <v>20</v>
       </c>
-      <c r="M87">
+      <c r="Q87">
         <v>400</v>
       </c>
-      <c r="O87" t="s">
+      <c r="S87" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>6</v>
       </c>
@@ -5624,16 +6687,28 @@
         <v>25</v>
       </c>
       <c r="L88">
+        <v>5.6</v>
+      </c>
+      <c r="M88">
+        <v>5.6</v>
+      </c>
+      <c r="N88" t="s">
+        <v>299</v>
+      </c>
+      <c r="O88">
+        <v>0.1</v>
+      </c>
+      <c r="P88">
         <v>20</v>
       </c>
-      <c r="M88">
+      <c r="Q88">
         <v>400</v>
       </c>
-      <c r="O88" t="s">
+      <c r="S88" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>6</v>
       </c>
@@ -5667,16 +6742,28 @@
         <v>25</v>
       </c>
       <c r="L89">
+        <v>5.6</v>
+      </c>
+      <c r="M89">
+        <v>5.6</v>
+      </c>
+      <c r="N89" t="s">
+        <v>299</v>
+      </c>
+      <c r="O89">
+        <v>0.1</v>
+      </c>
+      <c r="P89">
         <v>20</v>
       </c>
-      <c r="M89">
+      <c r="Q89">
         <v>400</v>
       </c>
-      <c r="O89" t="s">
+      <c r="S89" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>6</v>
       </c>
@@ -5710,16 +6797,28 @@
         <v>25</v>
       </c>
       <c r="L90">
+        <v>5.6</v>
+      </c>
+      <c r="M90">
+        <v>5.6</v>
+      </c>
+      <c r="N90" t="s">
+        <v>299</v>
+      </c>
+      <c r="O90">
+        <v>0.1</v>
+      </c>
+      <c r="P90">
         <v>179</v>
       </c>
-      <c r="M90">
+      <c r="Q90">
         <v>400</v>
       </c>
-      <c r="O90" t="s">
+      <c r="S90" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>6</v>
       </c>
@@ -5753,16 +6852,28 @@
         <v>25</v>
       </c>
       <c r="L91">
+        <v>5.6</v>
+      </c>
+      <c r="M91">
+        <v>5.6</v>
+      </c>
+      <c r="N91" t="s">
+        <v>299</v>
+      </c>
+      <c r="O91">
+        <v>0.1</v>
+      </c>
+      <c r="P91">
         <v>179</v>
       </c>
-      <c r="M91">
+      <c r="Q91">
         <v>400</v>
       </c>
-      <c r="O91" t="s">
+      <c r="S91" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>6</v>
       </c>
@@ -5796,16 +6907,28 @@
         <v>25</v>
       </c>
       <c r="L92">
+        <v>5.6</v>
+      </c>
+      <c r="M92">
+        <v>5.6</v>
+      </c>
+      <c r="N92" t="s">
+        <v>299</v>
+      </c>
+      <c r="O92">
+        <v>0.1</v>
+      </c>
+      <c r="P92">
         <v>179</v>
       </c>
-      <c r="M92">
+      <c r="Q92">
         <v>400</v>
       </c>
-      <c r="O92" t="s">
+      <c r="S92" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>6</v>
       </c>
@@ -5839,12 +6962,24 @@
         <v>25</v>
       </c>
       <c r="L93">
+        <v>5.6</v>
+      </c>
+      <c r="M93">
+        <v>5.6</v>
+      </c>
+      <c r="N93" t="s">
+        <v>299</v>
+      </c>
+      <c r="O93">
+        <v>0.1</v>
+      </c>
+      <c r="P93">
         <v>179</v>
       </c>
-      <c r="M93">
+      <c r="Q93">
         <v>400</v>
       </c>
-      <c r="O93" t="s">
+      <c r="S93" t="s">
         <v>119</v>
       </c>
     </row>

</xml_diff>